<commit_message>
refactor: P1 리뷰 반영 — Mechanism 중복정리(56)·Candidate 정예화(6)·Grip 카테고리·Coordinate System 시트
사용자 리뷰 피드백 반영:
- Mechanism 58→56: 의미 중복 통합(발 균형→회전 / Branch 분기문) +
  APT·PPT 'Late Wrist Set' 오통합(반대 원인) 분리 + 용어 정합(Vertical Arm Motion)
- Candidate 12→6: 반복성 있는 개념만 유지, 단일 출현(Clubhead Drag 등)은 '관찰 노드 대기 목록'으로 강등
- GRP → Grip: 약어 제거, 풀네임 카테고리
- Foot Pressure 축: Anterior/Posterior 유지(좌표계 일관성) + Forefoot/Rearfoot Alias
- DOH Coordinate System 시트 신설: Axis 마스터 레퍼런스(전 Object 재사용)
- P7 개선제안 갱신: Side Naming·Movement Environment 승격 승인 /
  Phase Pair·Prediction·Observed 태그 보류

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WzgekrgM9UsJ1Lha7AccVR
</commit_message>
<xml_diff>
--- a/DOH_P1.xlsx
+++ b/DOH_P1.xlsx
@@ -12,15 +12,16 @@
     <sheet name="Feature_Dictionary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Observation_Dictionary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Naming Rule" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Evidence Layer" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Evidence Matrix" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="DOH Setup Influence" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="DOH Candidate Concepts" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DOH Biomechanical Concepts" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="DOH Coaching Knowledge" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Derived Parameters" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="DOH Change Log" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Todo" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="DOH Coordinate System" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Evidence Layer" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Evidence Matrix" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DOH Setup Influence" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DOH Candidate Concepts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="DOH Biomechanical Concepts" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="DOH Coaching Knowledge" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Derived Parameters" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DOH Change Log" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Todo" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -798,13 +799,7 @@
 Limited Pelvic Motion Increases Dependence On Thorax Rotation.
 (골반 회전이 제한되면 흉곽 회전 의존도가 증가한다.)
  ↓
-Thorax Dominant Rotation (P4) [Candidate]
-Pelvis Tilt Anterior Excessive (P1)
- ↓
-Early Thoracic Extension Can Delay Natural Wrist Set.
-(조기 흉추 신전은 자연스러운 코킹 형성을 지연시킬 수 있다.)
- ↓
-Late Wrist Set (P2~P4) [예측·검증필요]</t>
+Thorax Dominant Rotation (P4) [Candidate]</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1351,7 @@
 [Pattern Dependent]
 Weak Grip Match (P1)
  ↓
-Reduced Forearm Support Promotes A Steeper Arm Motion.
+Reduced Forearm Support Promotes Vertical Arm Motion.
 (전완의 지지가 감소하여 팔이 더욱 수직적으로 움직인다.)
  ↓
 Lead Arm Lift (P2~P4) [예측·검증필요]
@@ -2017,8 +2012,8 @@
           <t>[High Confidence]
 Foot Pressure Anterior Excessive (P1)
  ↓
-Forward Balance Bias Reduces Rotational Freedom.
-(전방으로 치우친 균형은 회전의 자유도를 감소시킨다.)
+Excessive Foot Balance Bias Reduces Available Rotation.
+(중립을 벗어난 발 균형은 가용 회전량을 감소시킨다.)
  ↓
 Reduced Pelvis Rotation / Reduced Thorax Rotation (P4) [예측·검증필요]
 Foot Pressure Anterior Excessive (P1)
@@ -2035,8 +2030,8 @@
  ↓
 Steep Shaft (P4~P6) [예측·검증필요]
 ── Branch (분기) ──
-The Player Chooses A Different Balance Recovery Strategy.
-(선택된 균형 회복 전략이 이후 Chain을 결정한다.)
+The Player Chooses A Different Compensation Strategy During The Backswing.
+(백스윙에서 선택된 보상 전략이 이후 Chain을 결정한다.)
 Foot Pressure Anterior Excessive (P1)
  ↓
 The Player Shifts The Hips Rearward To Recover Balance.
@@ -2165,8 +2160,8 @@
 Inside Takeaway (P2) [예측·검증필요]
 Foot Pressure Posterior Excessive (P1)
  ↓
-Heel-Ward Balance Reduces Available Rotation.
-(후족부 균형은 가용 회전량을 감소시킨다.)
+Excessive Foot Balance Bias Reduces Available Rotation.
+(중립을 벗어난 발 균형은 가용 회전량을 감소시킨다.)
  ↓
 Reduced Pelvis Rotation / Reduced Thorax Rotation (P4) [예측·검증필요]
 [Pattern Dependent]
@@ -2287,8 +2282,8 @@
       <c r="B106" s="6" t="inlineStr">
         <is>
           <t>── Branch (분기) ──
-The Player Chooses A Different Pressure Strategy During The Backswing.
-(백스윙에서 선택된 압력 전략이 이후 Chain을 결정한다.)
+The Player Chooses A Different Compensation Strategy During The Backswing.
+(백스윙에서 선택된 보상 전략이 이후 Chain을 결정한다.)
 [High Confidence]
 Lead Pressure Excessive (P1)
  ↓
@@ -2366,6 +2361,280 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>First Found</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Repeated</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Example / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Flat Body Rotation</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>몸통이 수직 회전보다 수평 회전 성향을 더 많이 보이는 회전 패턴. 흉추 신전 부족과 함께 나타나며 팔이 과도하게 안쪽으로 이동하기 쉽다.</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>P1 – Pelvis Tilt Posterior Excessive</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr"/>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Posterior Tilt → Flat Body Rotation → Inside Takeaway / Deep Hands. 반복 시 Biomechanical Concept 승격 검토.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Grip Match</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>리드 손과 트레일 손의 그립 방향이 서로 생체역학적으로 대응하는 정도(Strong/Weak/Neutral Match). 관용/상위 개념.</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>P1 – Weak/Strong Grip Match</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Strong/Weak Grip Match Core Feature의 상위 개념(2 Feature에서 사용). Naming 관용명 유지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Arm Clearance</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>팔이 몸통과 간섭 없이 자연스럽게 움직일 수 있는 공간. 체형·흉곽 두께·셋업 자세에 영향.</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>P1 – Deep Thorax (Setup Influence)</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Deep Thorax → Reduced Arm Clearance → Lead Arm Lift/Outside. 여러 Anthropometry에서 반복.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Balance Recovery Strategy</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>초기 균형이 무너진 상태에서 반대 방향으로 압력·자세를 이동시켜 균형을 회복하려는 보상 전략.</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>P1 – Foot Pressure (AP)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Foot Pressure Anterior/Posterior 및 Lead Pressure의 Branch 분기 원인(3 Feature). 반복성 확인됨.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Compensatory Setup</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>신체 구조·가동성을 보상하기 위해 의도적으로 일반 기준과 다른 셋업을 사용하는 전략.</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>P1 – Asymmetrical Foot Angle</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>좌우 발각도 비대칭 등. ④ 계층: 체형형 vs 습관형 구분과 연결. P2~P8에서 반복 예상.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Movement Environment</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>P1 Setup이 정의하는, 특정 움직임이 발생하기 쉬운 초기 조건/움직임 편향(Initial Condition·Movement Bias). 확정 인과가 아닌 Prediction 대상.</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>P1 – 전체 Setup Feature</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Candidate (승격 검토중)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>DOH 해석 철학(Knowledge Structure). P1 전 13 Feature의 상위 프레임. ★사용자 승격 승인 — 반복성 확인 후 Knowledge Structure로 승격.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>── DOH Candidate Concepts ── (검증 대기 공간 / Holding Area) · 반복성 있는 개념만 유지(6개)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>⑤ 원칙: 새 Concept·해석 철학·Knowledge Structure·Feature화 애매 항목은 즉시 Feature화하지 않고 여기 먼저 등록. Repeated는 최초 등록 시 공백.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Promotion Rule: 3회 이상 반복 또는 2개 이상 Position(P1~P8)에서 재사용될 때 Feature/Biomechanical/Dictionary/Knowledge Structure 중 적절한 위치로 승격 검토.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>── 관찰 노드 대기 목록 (Concept 아님 · P2~P4 표준화 대기 · 단일 출현이라 Candidate 미등록) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Reverse Pivot — 다운스윙 보상 다양, P5~P7 검증 대상(관용명). / Flat·Steep Shaft (Backswing) — Shaft Plane 축, P4~P6 Observation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Excessive Hip Depth — Balance Recovery A 결과, P4 검증. / Balance Loss — P2~P4 검증. / Clubhead Drag — 현재 P1 단일 출현, P2~P4에서 반복되면 Candidate 승격 검토. / Thorax Dominant Rotation — 현재 APT 단일 출현, 반복 시 승격 검토.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>→ 위 노드들은 P2~P4 진행 중 반복 확인되면 Candidate Concepts로 정식 등록한다(살아남는 개념만 승격).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2560,13 +2829,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2927,22 +3196,44 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>── DOH Coaching Knowledge ── Feature/Mechanism/Observation만으로 설명하기 어려운 레슨 경험·조건부 해석·전략·예외.</t>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Terminology Alias</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Foot Pressure Anterior / Posterior</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>표준 축 용어는 Anterior(전족부)/Posterior(후족부)이며 Pelvis·Thorax·Spine과 좌표계를 공유한다. 회원 설명 시 가독성을 위해 Alias를 사용할 수 있다: Foot Pressure Anterior = Forefoot Pressure(앞꿈치/전족부 압력), Foot Pressure Posterior = Rearfoot Pressure(뒤꿈치/후족부 압력). Feature 이름·Knowledge Graph에는 Anterior/Posterior를 canonical로 사용한다.</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>AI는 Feature/Mechanism을 우선 사용하며, 충분히 설명되지 않을 때만 Coaching Knowledge를 참고해 설명·피드백·질문·전략을 생성한다.</t>
+          <t>── DOH Coaching Knowledge ── Feature/Mechanism/Observation만으로 설명하기 어려운 레슨 경험·조건부 해석·전략·예외.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>AI는 Feature/Mechanism을 우선 사용하며, 충분히 설명되지 않을 때만 Coaching Knowledge를 참고해 설명·피드백·질문·전략을 생성한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>※ Coaching Knowledge는 Observation이 아니며 Feature를 생성하지 않는다. AI의 최종 판단 근거가 아니라 Explanation/Coaching/Strategy/Exception 제공용이다.</t>
         </is>
@@ -2953,7 +3244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3022,13 +3313,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3061,12 +3352,12 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Mechanism 카테고리 GRP 신설</t>
+          <t>Mechanism 카테고리 Grip 신설</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Grip(양손 그립 조합)이 팔 연결성·페이스·코킹에 미치는 영향 Mechanism. P7의 8개 카테고리에 추가(PST 신설 선례와 동일 방식).</t>
+          <t>Grip(양손 그립 조합)이 팔 연결성·페이스·코킹에 미치는 영향 Mechanism. P7의 8개 카테고리에 추가(PST 신설 선례와 동일 방식). ※약어 없이 풀네임 'Grip' 사용(사용자 선호). P7 카테고리는 LOCK이라 약어 유지, 차기 Refactoring에서 풀네임 통일 검토.</t>
         </is>
       </c>
     </row>
@@ -3095,12 +3386,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Coordinate 축 신설</t>
+          <t>DOH Coordinate System 시트 신설</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure AP(Anterior=전족부/Posterior=후족부) — Target Line의 Forward/Backward 및 Lateral(Lead/Trail)과 독립 축으로 등록(혼동 방지).</t>
+          <t>Axis 마스터 레퍼런스(Anterior/Posterior·Superior/Inferior·Medial/Lateral·Internal/External 등) + Alias + Used By. 전 Object 좌표계 통일 → P2~P8에서 축 재정의 불필요. (사용자 제안 채택)</t>
         </is>
       </c>
     </row>
@@ -3112,12 +3403,12 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Feature Dictionary 13</t>
+          <t>Coordinate 축 신설 + Alias</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>P1 Core Feature 13개 등록(Feature_Dictionary 시트). 모두 Information Gain 충족.</t>
+          <t>Foot Pressure AP(Anterior=전족부/Posterior=후족부) — Target Line의 Forward/Backward 및 Lateral(Lead/Trail)과 독립 축. ★표준 축은 Anterior/Posterior 유지(Pelvis·Thorax·Spine과 좌표계 공유). 가독성 Alias: Anterior=Forefoot, Posterior=Rearfoot(Coaching Knowledge 등록). (사용자 승인)</t>
         </is>
       </c>
     </row>
@@ -3129,114 +3420,114 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Observation Dictionary 13</t>
+          <t>Feature Dictionary 13</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>P1 표준 관찰문장 13개 + Coordinate Reference 등록.</t>
+          <t>P1 Core Feature 13개 등록(Feature_Dictionary 시트). 모두 Information Gain 충족.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>DOH Mechanism Added</t>
+          <t>DOH Dictionary Added</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>P1 Mechanism 62문장</t>
+          <t>Observation Dictionary 13</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Mechanism_Dictionary 시트. 대부분 P1 신규(Setup→Possible Observation, Prediction). ★재사용 Node: 'Vertical Arm Motion Promotes A Steeper Shaft Plane.'(Weak Grip Match/Toe-In 공통). ★Branch 분기 표준문장 2개(균형회복/압력전략).</t>
+          <t>P1 표준 관찰문장 13개 + Coordinate Reference 등록.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>DOH Coaching Knowledge Added</t>
+          <t>DOH Mechanism Added</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Coaching 15항목</t>
+          <t>P1 Mechanism 56문장</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>그립·Anthropometry·압력분포·Toe-Out/In·Lead Pressure·Compensatory Foot Angle·Lift The Ball·Arm Dominant·Structure vs Habit(계층 판단) 등 정리·표준화(Category/Topic/Knowledge/Confidence).</t>
+          <t>Mechanism_Dictionary 시트(중복 검토 완료, 58→56). 대부분 P1 신규(Setup→Possible Observation, Prediction). ★재사용 Node: 'Vertical Arm Motion Promotes A Steeper Shaft Plane.' · 'Excessive Foot Balance Bias Reduces Available Rotation.'(Anterior/Posterior 통합) · Branch 표준문장 'The Player Chooses A Different Compensation Strategy During The Backswing.'(통합).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>DOH Candidate Concepts Added</t>
+          <t>DOH Mechanism 정리</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Candidate 12개</t>
+          <t>중복 통합 3건</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Flat Body Rotation·Grip Match·Clubhead Drag·Arm Clearance·Balance Recovery Strategy·Compensatory Setup·Thorax Dominant Rotation·Movement Environment(해석철학) + downstream candidate-observation(Reverse Pivot·Flat/Steep Shaft·Excessive Hip Depth·Balance Loss). Repeated 공백(선등록).</t>
+          <t>①발 균형→회전 2문장 통합 ②Branch 분기 2문장 통합 ③APT/PPT 'Late Wrist Set' 오통합(반대 원인) 분리 후 APT 저가치 체인 제거 ④'Steeper Arm Motion'→'Vertical Arm Motion' 용어 정합. shoulder/elbow→Outside 등은 Object 상이로 유지.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>DOH Biomechanical Added</t>
+          <t>DOH Coaching Knowledge Added</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Biomech 4항목 추가</t>
+          <t>Coaching 16항목</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Thoracic Extension·Hip Rotation(In/Ext)·Lumbar Lordosis·Center Of Pressure — P1 Mechanism 반복 근거로 등록(기존 Hip Hinge·Swing Radius 유지).</t>
+          <t>그립·Anthropometry·압력분포·Toe-Out/In·Lead Pressure·Compensatory Foot Angle·Lift The Ball·Arm Dominant·Structure vs Habit·Foot Pressure Alias 등 정리·표준화(Category/Topic/Knowledge/Confidence).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>규칙 적용</t>
+          <t>DOH Candidate Concepts Added</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Fat/Thin 제거</t>
+          <t>Candidate 6개 (반복성 있는 것만)</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>초안 Lead Pressure Chain의 'Fat/Thin'은 Evidence Layer이므로 Feature Chain에서 제거하고 Evidence Matrix에서만 관리(P7 Evidence 규칙 준수).</t>
+          <t>Flat Body Rotation·Grip Match·Arm Clearance·Balance Recovery Strategy·Compensatory Setup·Movement Environment. Repeated 공백(선등록). 단일 출현(Clubhead Drag·Thorax Dominant Rotation 등)은 '관찰 노드 대기 목록'으로 강등 — P2~P4 반복 확인 후 승격.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>규칙 적용</t>
+          <t>DOH Biomechanical Added</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Grip 모델링</t>
+          <t>Biomech 4항목 추가</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>단일 Strong/Weak Grip은 Core Feature化하지 않고 Setup Influence+Coaching으로 관리. Strong/Weak Grip Match만 Core(Information Gain). (사용자 승인)</t>
+          <t>Thoracic Extension·Hip Rotation(In/Ext)·Lumbar Lordosis·Center Of Pressure — P1 Mechanism 반복 근거로 등록(기존 Hip Hinge·Swing Radius 유지).</t>
         </is>
       </c>
     </row>
@@ -3248,89 +3539,123 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Anthropometry/Mobility 분리</t>
+          <t>Fat/Thin 제거</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Long Arm·Deep Thorax·Limited Hip IR 등은 Feature가 아니라 Setup Influence의 Reference로만 관리(④ 계층 분리).</t>
+          <t>초안 Lead Pressure Chain의 'Fat/Thin'은 Evidence Layer이므로 Feature Chain에서 제거하고 Evidence Matrix에서만 관리(P7 Evidence 규칙 준수).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>── P7 Standard 개선 제안 (참고용, 미변경) ──</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="7" t="inlineStr"/>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>규칙 적용</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Grip 모델링</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>단일 Strong/Weak Grip은 Core Feature化하지 않고 Setup Influence+Coaching으로 관리. Strong/Weak Grip Match만 Core(Information Gain). (사용자 승인)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>제안 1</t>
+          <t>규칙 적용</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Naming Rule에 'Side 배치 관례' 명문화</t>
+          <t>Anthropometry/Mobility 분리</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>P7은 Lead/Trail Side 배치 규칙이 암묵적. P1에서 'Object Axis [Side] [Attribute]' 관례를 명문화했으므로, 차기 Dictionary Refactoring 시 P7 Naming Rule에도 역반영 제안. (현재 P7 미변경)</t>
+          <t>Long Arm·Deep Thorax·Limited Hip IR 등은 Feature가 아니라 Setup Influence의 Reference로만 관리(④ 계층 분리).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>제안 2</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Phase-Distinguished Pair 명시 필드</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Lead Pressure Excessive (P1)↔(P7)처럼 동일 Object/Axis·다른 Phase Feature가 늘어남. Feature Dictionary에 'Phase Pair' 컬럼 추가를 제안(교차 Phase 추론 강화). (현재 P7 미변경)</t>
-        </is>
-      </c>
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>── P7 Standard 개선 제안 (참고용, 미변경) ──</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr"/>
+      <c r="C16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>제안 3</t>
+          <t>제안 1 — ★승인</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Prediction vs Causation 태그</t>
+          <t>Naming Rule에 'Side 배치 관례' 명문화</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>P1은 Prediction Knowledge, P7 원인추정은 상대적으로 확정도가 높음. Chain에 [Prediction]/[Observed] 성격 태그를 추가하면 AI가 확신도를 구분하기 쉬움. (제안만, P7 미변경)</t>
+          <t>P1에서 'Object Axis [Side] [Attribute]' 관례를 명문화. 사용자 승인 — 차기 Dictionary Refactoring 시 P7 Naming Rule에도 역반영 예정. (현재 P7 미변경)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>제안 4</t>
+          <t>제안 2 — 보류</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Movement Environment를 Knowledge Structure로 승격 검토</t>
+          <t>Movement Environment를 Knowledge Structure로 승격</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>P1 전반을 관통하는 'Setup=Movement Environment' 프레임을 반복성 확인 후 DOH Knowledge Structure로 승격 검토(현재 Candidate).</t>
+          <t>'Setup=Movement Environment' 프레임을 Knowledge Structure로 승격 검토. ★사용자 승인 — 반복성 확인(P2~P4) 후 정식 승격. (현재 Candidate 유지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>제안 3 — 보류</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Phase-Distinguished Pair 명시 필드</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>사용자 보류: Knowledge Graph가 자동 연결해야 하며 문서에 Pair를 쓰면 중복 관리가 됨. P2~P4 진행 후 재판단. (미반영)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>제안 4 — 보류</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Prediction vs Observed 태그</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>사용자 보류: P1 자체가 Prediction, P7이 Observation이므로 별도 태그 불필요할 수 있음. P2~P4 진행 후 재판단. (미반영)</t>
         </is>
       </c>
     </row>
@@ -3339,13 +3664,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3384,7 +3709,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Naming Rule(P1) + Axis 확정(Foot/Shoulder/Elbow/Pelvis/Shaft/Grip) + GRP 카테고리</t>
+          <t>Naming Rule(P1) + Axis 확정(Foot/Shoulder/Elbow/Pelvis/Shaft/Grip) + Grip 카테고리</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -3406,7 +3731,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Feature_Dictionary 구축(Core 13)</t>
+          <t>DOH Coordinate System 시트(Axis 마스터 레퍼런스 + Alias)</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -3416,7 +3741,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Information Gain 충족 확인.</t>
+          <t>전 Object 좌표계 통일. P2~P8 재사용. (사용자 제안)</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3753,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Observation_Dictionary(표준 관찰문장 + Coordinate)</t>
+          <t>Feature_Dictionary 구축(Core 13)</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -3436,7 +3761,11 @@
           <t>done</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Information Gain 충족 확인.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -3446,7 +3775,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Mechanism_Dictionary(재사용 우선, 신규 최소)</t>
+          <t>Observation_Dictionary(표준 관찰문장 + Coordinate)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -3454,11 +3783,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>62문장. ★재사용 Node/Branch 표준문장 표시.</t>
-        </is>
-      </c>
+      <c r="D5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -3468,7 +3793,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Setup Influence(Setup/Anthropometry/Mobility → Prediction)</t>
+          <t>Mechanism_Dictionary(재사용 우선, 신규 최소)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3478,7 +3803,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>계층 분리 반영.</t>
+          <t>56문장(중복 검토·통합 완료, 58→56). ★재사용 Node/Branch 표준문장 표시.</t>
         </is>
       </c>
     </row>
@@ -3490,7 +3815,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Candidate Concepts 통합 + 신규 등록</t>
+          <t>Setup Influence(Setup/Anthropometry/Mobility → Prediction)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -3500,7 +3825,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>중복 시트 통합. Repeated 공백.</t>
+          <t>계층 분리 반영.</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3837,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Biomechanical Concepts 확장</t>
+          <t>Candidate Concepts 통합 + 신규 등록</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -3522,7 +3847,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Thoracic Extension 등 4항목 추가.</t>
+          <t>중복 시트 통합. Repeated 공백.</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3859,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Coaching Knowledge 보존·표준화</t>
+          <t>Biomechanical Concepts 확장</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -3544,7 +3869,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>15항목. Category/Topic/Knowledge/Confidence.</t>
+          <t>Thoracic Extension 등 4항목 추가.</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3881,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Evidence Layer/Matrix 구조(별점 보류)</t>
+          <t>Coaching Knowledge 보존·표준화</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -3566,19 +3891,19 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>P1 간접 연결 특성 명시.</t>
+          <t>15항목. Category/Topic/Knowledge/Confidence.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>P1 메인 시트: Core 13 Feature 6-섹션</t>
+          <t>Evidence Layer/Matrix 구조(별점 보류)</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -3588,7 +3913,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Dictionary 기준 문장 사용. Movement Environment 관점.</t>
+          <t>P1 간접 연결 특성 명시.</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3925,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>규칙 적용: Chain 종료·Branch Mechanism·Confidence 3단계·Family·Fat/Thin 제거</t>
+          <t>P1 메인 시트: Core 13 Feature 6-섹션</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -3608,7 +3933,11 @@
           <t>done</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr"/>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Dictionary 기준 문장 사용. Movement Environment 관점.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -3618,7 +3947,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>DOH Change Log(Added 정리 + P7 개선 제안)</t>
+          <t>규칙 적용: Chain 종료·Branch Mechanism·Confidence 3단계·Family·Fat/Thin 제거</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -3626,31 +3955,27 @@
           <t>done</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>규칙 ⑥.</t>
-        </is>
-      </c>
+      <c r="D13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Evidence Matrix 별점 일괄 부여</t>
+          <t>DOH Change Log(Added 정리 + P7 개선 제안)</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>todo</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>P1~P8 설계 완료 후 별도 세션.</t>
+          <t>규칙 ⑥.</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3987,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>HTML/JSON 변환</t>
+          <t>Evidence Matrix 별점 일괄 부여</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -3672,23 +3997,45 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>P1~P8 LOCK 후 일괄.</t>
+          <t>P1~P8 설계 완료 후 별도 세션.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>HTML/JSON 변환</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>P1~P8 LOCK 후 일괄.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
           <t>참고</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>작업 순서</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr"/>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Dictionary → Feature 6-섹션 → Evidence 별점 → HTML/JSON. 동일 의미=동일 문장.</t>
         </is>
@@ -3705,7 +4052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4176,27 +4523,23 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Early Thoracic Extension Can Delay Natural Wrist Set.</t>
+          <t>Reduced Thoracic Extension Can Delay Natural Wrist Set.</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>조기 흉추 신전은 자연스러운 코킹 형성을 지연시킬 수 있다.</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Reduced Thoracic Extension Can Delay Natural Wrist Set.</t>
-        </is>
-      </c>
+          <t>흉추 신전 부족은 자연스러운 코킹 형성을 지연시킬 수 있다.</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr"/>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Pelvis Tilt Anterior Excessive (P1)</t>
+          <t>Pelvis Tilt Posterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. ★Thoracic Extension→Late Wrist Set 표준(전/후경 통합 대표).</t>
+          <t>P1 신규. Posterior Tilt→Late Wrist Set→Across The Line. (Anterior의 '조기 신전'과는 반대 원인이라 별개 Mechanism)</t>
         </is>
       </c>
     </row>
@@ -4548,23 +4891,27 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Forward Balance Bias Reduces Rotational Freedom.</t>
+          <t>Excessive Foot Balance Bias Reduces Available Rotation.</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>전방으로 치우친 균형은 회전의 자유도를 감소시킨다.</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr"/>
+          <t>중립을 벗어난 발 균형(전족부/후족부)은 가용 회전량을 감소시킨다.</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Forward Balance Bias Reduces Rotational Freedom. / Heel-Ward Balance Reduces Available Rotation.</t>
+        </is>
+      </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure Anterior Excessive (P1)</t>
+          <t>Foot Pressure Anterior Excessive (P1) / Foot Pressure Posterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Reduced Rotation.</t>
+          <t>★P1 재사용 Node — Anterior/Posterior 공통(2개 통합).</t>
         </is>
       </c>
     </row>
@@ -4576,51 +4923,51 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Heel-Ward Balance Reduces Available Rotation.</t>
+          <t>Excessive Lateral Motion Reduces Thorax Rotation.</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>후족부 균형은 가용 회전량을 감소시킨다.</t>
+          <t>과도한 좌우 이동은 흉곽 회전을 감소시킨다.</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr"/>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure Posterior Excessive (P1)</t>
+          <t>Lead Pressure Excessive (P1)</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Reduced Rotation.</t>
+          <t>P1 신규. Sway→Closed Thorax At Top. (P7 Slide 계열과 의미 호환)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>ROT</t>
+          <t>PST</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Excessive Lateral Motion Reduces Thorax Rotation.</t>
+          <t>An Excessive Lumbar Arch Restricts Efficient Hip Hinge During The Backswing.</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>과도한 좌우 이동은 흉곽 회전을 감소시킨다.</t>
+          <t>과도한 요추 전만은 백스윙에서 효율적인 힙힌지를 제한한다.</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr"/>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Lead Pressure Excessive (P1)</t>
+          <t>Pelvis Tilt Anterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. Sway→Closed Thorax At Top. (P7 Slide 계열과 의미 호환)</t>
+          <t>P1 신규. →Limited Hip Hinge.</t>
         </is>
       </c>
     </row>
@@ -4632,12 +4979,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>An Excessive Lumbar Arch Restricts Efficient Hip Hinge During The Backswing.</t>
+          <t>Early Thoracic Extension Tilts The Upper Body Rearward.</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>과도한 요추 전만은 백스윙에서 효율적인 힙힌지를 제한한다.</t>
+          <t>조기 흉추 신전이 상체를 뒤로 기울게 만든다.</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr"/>
@@ -4648,7 +4995,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Limited Hip Hinge.</t>
+          <t>P1 신규. →Reverse Pivot(패턴).</t>
         </is>
       </c>
     </row>
@@ -4660,12 +5007,12 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Early Thoracic Extension Tilts The Upper Body Rearward.</t>
+          <t>Early Thoracic Extension Promotes Vertical Arm Motion.</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>조기 흉추 신전이 상체를 뒤로 기울게 만든다.</t>
+          <t>조기 흉추 신전은 팔의 수직 움직임을 증가시킨다.</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr"/>
@@ -4676,7 +5023,7 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Reverse Pivot(패턴).</t>
+          <t>P1 신규. →Lead Arm Lift(패턴).</t>
         </is>
       </c>
     </row>
@@ -4688,12 +5035,12 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Early Thoracic Extension Promotes Vertical Arm Motion.</t>
+          <t>Early Thoracic Extension Reduces Hand Depth During The Backswing.</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>조기 흉추 신전은 팔의 수직 움직임을 증가시킨다.</t>
+          <t>조기 흉추 신전은 백스윙에서 손의 깊이를 감소시킨다.</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr"/>
@@ -4704,7 +5051,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Lead Arm Lift(패턴).</t>
+          <t>P1 신규. →Shallow Hand Depth.</t>
         </is>
       </c>
     </row>
@@ -4716,23 +5063,23 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Early Thoracic Extension Reduces Hand Depth During The Backswing.</t>
+          <t>The Player Tends To Sit Excessively During The Backswing.</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>조기 흉추 신전은 백스윙에서 손의 깊이를 감소시킨다.</t>
+          <t>백스윙에서 과도하게 앉는 움직임이 나타나기 쉽다.</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr"/>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Pelvis Tilt Anterior Excessive (P1)</t>
+          <t>Pelvis Tilt Posterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Shallow Hand Depth.</t>
+          <t>P1 신규. →Excessive Knee Flexion(패턴).</t>
         </is>
       </c>
     </row>
@@ -4744,51 +5091,51 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>The Player Tends To Sit Excessively During The Backswing.</t>
+          <t>A Steeper Shaft Reduces Hand Depth At The Top.</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>백스윙에서 과도하게 앉는 움직임이 나타나기 쉽다.</t>
+          <t>가파른 샤프트는 백스윙 탑에서 손의 깊이를 감소시킨다.</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr"/>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Pelvis Tilt Posterior Excessive (P1)</t>
+          <t>Weak Grip Match (P1)</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Excessive Knee Flexion(패턴).</t>
+          <t>P1 신규. Steep Shaft→Shallow Hand Depth.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>PST</t>
+          <t>SPC</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>A Steeper Shaft Reduces Hand Depth At The Top.</t>
+          <t>Excessive Elbow Flexion Reduces The Swing Radius.</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>가파른 샤프트는 백스윙 탑에서 손의 깊이를 감소시킨다.</t>
+          <t>과도한 팔꿈치 굴곡이 스윙 반경을 감소시킨다.</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr"/>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Weak Grip Match (P1)</t>
+          <t>Elbow Flexion Trail Excessive (P1)</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. Steep Shaft→Shallow Hand Depth.</t>
+          <t>P1 신규. →Small Swing Arc. (Biomech: Swing Radius)</t>
         </is>
       </c>
     </row>
@@ -4800,23 +5147,23 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Excessive Elbow Flexion Reduces The Swing Radius.</t>
+          <t>The Hands Travel Deeper Around The Thorax.</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>과도한 팔꿈치 굴곡이 스윙 반경을 감소시킨다.</t>
+          <t>손이 흉곽을 따라 더욱 깊게 이동한다.</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr"/>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Elbow Flexion Trail Excessive (P1)</t>
+          <t>Pelvis Tilt Posterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Small Swing Arc. (Biomech: Swing Radius)</t>
+          <t>P1 신규. Flat Body Rotation→Deep Hands.</t>
         </is>
       </c>
     </row>
@@ -4828,12 +5175,12 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>The Hands Travel Deeper Around The Thorax.</t>
+          <t>The Hands Continue Moving Behind The Body.</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>손이 흉곽을 따라 더욱 깊게 이동한다.</t>
+          <t>손이 몸 뒤쪽으로 계속 이동한다.</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr"/>
@@ -4844,7 +5191,7 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. Flat Body Rotation→Deep Hands.</t>
+          <t>P1 신규. →Hands Behind Body(패턴).</t>
         </is>
       </c>
     </row>
@@ -4856,51 +5203,51 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>The Hands Continue Moving Behind The Body.</t>
+          <t>Reduced Arm Width Promotes Deeper Hand Travel.</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>손이 몸 뒤쪽으로 계속 이동한다.</t>
+          <t>팔의 폭이 감소하면서 손이 몸 안쪽으로 더 깊게 이동하기 쉽다.</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr"/>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Pelvis Tilt Posterior Excessive (P1)</t>
+          <t>Strong Grip Match (P1)</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Hands Behind Body(패턴).</t>
+          <t>P1 신규. →Deep Hands.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>SPC</t>
+          <t>PRS</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Reduced Arm Width Promotes Deeper Hand Travel.</t>
+          <t>Forward Balance Bias Shifts Pressure Toward The Toes.</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>팔의 폭이 감소하면서 손이 몸 안쪽으로 더 깊게 이동하기 쉽다.</t>
+          <t>전방으로 치우친 균형은 압력을 전족부 방향으로 이동시킨다.</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr"/>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>Strong Grip Match (P1)</t>
+          <t>Pelvis Tilt Anterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Deep Hands.</t>
+          <t>P1 신규. →Foot Pressure Anterior.</t>
         </is>
       </c>
     </row>
@@ -4912,23 +5259,23 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Forward Balance Bias Shifts Pressure Toward The Toes.</t>
+          <t>Pressure Remains On The Lead Side During The Backswing.</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>전방으로 치우친 균형은 압력을 전족부 방향으로 이동시킨다.</t>
+          <t>백스윙 동안 압력이 리드측에 남아 있다.</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr"/>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Pelvis Tilt Anterior Excessive (P1)</t>
+          <t>Lead Pressure Excessive (P1)</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Foot Pressure Anterior.</t>
+          <t>P1 신규. →Reverse Pivot(Hold Strategy).</t>
         </is>
       </c>
     </row>
@@ -4940,51 +5287,51 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Pressure Remains On The Lead Side During The Backswing.</t>
+          <t>Rearward Balance Reduces Postural Stability.</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>백스윙 동안 압력이 리드측에 남아 있다.</t>
+          <t>후방 균형은 자세 안정성을 감소시킨다.</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr"/>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Lead Pressure Excessive (P1)</t>
+          <t>Foot Pressure Posterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Reverse Pivot(Hold Strategy).</t>
+          <t>P1 신규. →Balance Loss(Candidate).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>PRS</t>
+          <t>CMP</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Rearward Balance Reduces Postural Stability.</t>
+          <t>The Body Tilts Rearward To Maintain Balance.</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>후방 균형은 자세 안정성을 감소시킨다.</t>
+          <t>균형을 유지하기 위해 몸이 뒤로 기울어지는 보상이 나타날 수 있다.</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr"/>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure Posterior Excessive (P1)</t>
+          <t>Shoulder Height Trail High (P1)</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Balance Loss(Candidate).</t>
+          <t>P1 신규. →Reverse Pivot(보상).</t>
         </is>
       </c>
     </row>
@@ -4996,23 +5343,23 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>The Body Tilts Rearward To Maintain Balance.</t>
+          <t>The Player May Lift The Lead Arm To Prevent The Club From Moving Too Far Inside.</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>균형을 유지하기 위해 몸이 뒤로 기울어지는 보상이 나타날 수 있다.</t>
+          <t>클럽이 과도하게 안쪽으로 이동하는 것을 막기 위해 리드암을 들어 올리는 보상이 나타날 수 있다.</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr"/>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Shoulder Height Trail High (P1)</t>
+          <t>Elbow Flexion Trail Excessive (P1)</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Reverse Pivot(보상).</t>
+          <t>P1 신규. →Lead Arm Lift→Disconnected(보상).</t>
         </is>
       </c>
     </row>
@@ -5024,23 +5371,23 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>The Player May Lift The Lead Arm To Prevent The Club From Moving Too Far Inside.</t>
+          <t>The Player Shifts The Hips Rearward To Recover Balance.</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>클럽이 과도하게 안쪽으로 이동하는 것을 막기 위해 리드암을 들어 올리는 보상이 나타날 수 있다.</t>
+          <t>균형을 회복하기 위해 엉덩이를 뒤로 빼며 공간을 확보한다.</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr"/>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>Elbow Flexion Trail Excessive (P1)</t>
+          <t>Foot Pressure Anterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Lead Arm Lift→Disconnected(보상).</t>
+          <t>P1 신규. Balance Recovery A→Excessive Hip Depth(Candidate).</t>
         </is>
       </c>
     </row>
@@ -5052,12 +5399,12 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>The Player Shifts The Hips Rearward To Recover Balance.</t>
+          <t>The Player Shifts Pressure Rearward To Recover Balance During The Backswing.</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>균형을 회복하기 위해 엉덩이를 뒤로 빼며 공간을 확보한다.</t>
+          <t>백스윙에서 균형을 회복하려 압력을 뒤꿈치로 이동시킨다.</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr"/>
@@ -5068,7 +5415,7 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. Balance Recovery A→Excessive Hip Depth(Candidate).</t>
+          <t>P1 신규. Balance Recovery B→Heel Pressure At Top.</t>
         </is>
       </c>
     </row>
@@ -5080,23 +5427,23 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>The Player Shifts Pressure Rearward To Recover Balance During The Backswing.</t>
+          <t>The Player Shifts Pressure Forward To Recover Balance During The Backswing.</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>백스윙에서 균형을 회복하려 압력을 뒤꿈치로 이동시킨다.</t>
+          <t>백스윙에서 균형을 회복하려 압력을 전족부로 이동시킨다.</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr"/>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure Anterior Excessive (P1)</t>
+          <t>Foot Pressure Posterior Excessive (P1)</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. Balance Recovery B→Heel Pressure At Top.</t>
+          <t>P1 신규. →Toe Pressure During Backswing(보상).</t>
         </is>
       </c>
     </row>
@@ -5108,23 +5455,23 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>The Player Shifts Pressure Forward To Recover Balance During The Backswing.</t>
+          <t>The Player Attempts To Recenter Pressure During The Backswing.</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>백스윙에서 균형을 회복하려 압력을 전족부로 이동시킨다.</t>
+          <t>백스윙에서 압력을 정상 위치로 되돌리려 한다.</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr"/>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure Posterior Excessive (P1)</t>
+          <t>Lead Pressure Excessive (P1)</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. →Toe Pressure During Backswing(보상).</t>
+          <t>P1 신규. Recenter Strategy→Sway.</t>
         </is>
       </c>
     </row>
@@ -5136,99 +5483,107 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>The Player Attempts To Recenter Pressure During The Backswing.</t>
+          <t>The Player Chooses A Different Compensation Strategy During The Backswing.</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>백스윙에서 압력을 정상 위치로 되돌리려 한다.</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr"/>
+          <t>백스윙에서 선택된 보상 전략이 이후 Chain을 결정한다.</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>The Player Chooses A Different Balance Recovery Strategy. / The Player Chooses A Different Pressure Strategy During The Backswing.</t>
+        </is>
+      </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Lead Pressure Excessive (P1)</t>
+          <t>Foot Pressure Anterior Excessive (P1) / Lead Pressure Excessive (P1)</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. Recenter Strategy→Sway.</t>
+          <t>★P1 Branch 분기 표준 문장(2개 통합). P7 'The Chosen Compensation Strategy Determines The Subsequent Chain.' 계열.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>CMP</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>The Player Chooses A Different Balance Recovery Strategy.</t>
+          <t>A Weak Grip Match Reduces Natural Arm Connection.</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>선택된 균형 회복 전략이 이후 Chain을 결정한다.</t>
+          <t>양손의 위크 그립 조합은 자연스러운 팔 연결성을 감소시킨다.</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr"/>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure Anterior Excessive (P1)</t>
+          <t>Weak Grip Match (P1)</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>★P1 Branch 분기 원인 표준 문장(균형 회복).</t>
+          <t>★P1 신규 카테고리 Grip. →Trail Elbow Out.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>CMP</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>The Player Chooses A Different Pressure Strategy During The Backswing.</t>
+          <t>The Clubface Is More Difficult To Square Naturally.</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>백스윙에서 선택된 압력 전략이 이후 Chain을 결정한다.</t>
+          <t>클럽페이스를 자연스럽게 스퀘어하기 어려운 구조가 된다.</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr"/>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Lead Pressure Excessive (P1)</t>
+          <t>Weak Grip Match (P1)</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>★P1 Branch 분기 원인 표준 문장(압력 전략).</t>
+          <t>P1 신규(Grip). →Club Face Open At Takeaway.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>GRP</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>A Weak Grip Match Reduces Natural Arm Connection.</t>
+          <t>Reduced Forearm Support Promotes Vertical Arm Motion.</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>양손의 위크 그립 조합은 자연스러운 팔 연결성을 감소시킨다.</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="inlineStr"/>
+          <t>전완의 지지가 감소하여 팔이 더욱 수직적으로 움직인다.</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Reduced Forearm Support Promotes A Steeper Arm Motion.</t>
+        </is>
+      </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
           <t>Weak Grip Match (P1)</t>
@@ -5236,24 +5591,24 @@
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>★P1 신규 카테고리 GRP. →Trail Elbow Out.</t>
+          <t>P1 신규(Grip). →Lead Arm Lift. 'Vertical Arm Motion' 공통 Node에 정렬.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>GRP</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>The Clubface Is More Difficult To Square Naturally.</t>
+          <t>The Lead Wrist Tends To Extend At The Top.</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>클럽페이스를 자연스럽게 스퀘어하기 어려운 구조가 된다.</t>
+          <t>백스윙 탑에서 리드 손목이 커핑되기 쉬워진다.</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr"/>
@@ -5264,152 +5619,103 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>P1 신규(GRP). →Club Face Open At Takeaway.</t>
+          <t>P1 신규(Grip). →Lead Wrist Extension(패턴).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>GRP</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Reduced Forearm Support Promotes A Steeper Arm Motion.</t>
+          <t>A Strong Grip Match Restricts Natural Trail Arm Folding.</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>전완의 지지가 감소하여 팔이 더욱 수직적으로 움직인다.</t>
+          <t>양손의 스트롱 그립 조합은 트레일 팔의 자연스러운 굴곡을 제한할 수 있다.</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr"/>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>Weak Grip Match (P1)</t>
+          <t>Strong Grip Match (P1)</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>P1 신규(GRP). →Lead Arm Lift.</t>
+          <t>P1 신규(Grip). →Late Trail Elbow Flexion.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>GRP</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>The Lead Wrist Tends To Extend At The Top.</t>
+          <t>A Strong Grip Match Can Delay Natural Wrist Set.</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>백스윙 탑에서 리드 손목이 커핑되기 쉬워진다.</t>
+          <t>양손의 스트롱 그립 조합은 자연스러운 코킹 형성을 지연시킬 수 있다.</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr"/>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Weak Grip Match (P1)</t>
+          <t>Strong Grip Match (P1)</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>P1 신규(GRP). →Lead Wrist Extension(패턴).</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>GRP</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>A Strong Grip Match Restricts Natural Trail Arm Folding.</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr">
-        <is>
-          <t>양손의 스트롱 그립 조합은 트레일 팔의 자연스러운 굴곡을 제한할 수 있다.</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="inlineStr"/>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>Strong Grip Match (P1)</t>
-        </is>
-      </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>P1 신규(GRP). →Late Trail Elbow Flexion.</t>
+          <t>P1 신규(Grip). →Late Wrist Set.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>GRP</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>A Strong Grip Match Can Delay Natural Wrist Set.</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>양손의 스트롱 그립 조합은 자연스러운 코킹 형성을 지연시킬 수 있다.</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr"/>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>Strong Grip Match (P1)</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>P1 신규(GRP). →Late Wrist Set.</t>
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>── DOH P1 Mechanism Dictionary ── (총 56문장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>③ 원칙: 동일 Mechanism 반복 시 재사용 우선. 새 Mechanism은 기존 Dictionary로 설명 불가할 때만 추가.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>── DOH P1 Mechanism Dictionary ──</t>
+          <t>★재사용 Node: 'Vertical Arm Motion Promotes A Steeper Shaft Plane.'(Weak Grip Match/Toe-In) · 'Excessive Foot Balance Bias Reduces Available Rotation.'(Anterior/Posterior) · Branch 표준문장(Anterior/Lead Pressure).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>③ 원칙: 동일 Mechanism 반복 시 재사용 우선. 새 Mechanism은 기존 Dictionary로 설명 불가할 때만 추가.</t>
+          <t>★신규 카테고리 Grip: P1에서 신설(풀네임). P7 카테고리(ROT/PRS/ARM/CLB/SPC/LOD/CMP/PST)에 추가. → Change Log 참조.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>★재사용 Node: 'Vertical Arm Motion Promotes A Steeper Shaft Plane.' — Weak Grip Match / Toe-In 공통 사용.</t>
+          <t>중복 검토 완료: 의미 중복 2쌍 통합(발 균형→회전 / Branch 문장), APT-PPT 'Late Wrist Set' 오통합 분리(반대 원인), 'Steeper Arm Motion'→'Vertical Arm Motion' 정합. shoulder/elbow→Outside 등은 Object 상이로 유지.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
-        <is>
-          <t>★신규 카테고리 GRP(Grip): P1에서 신설. P7 카테고리(ROT/PRS/ARM/CLB/SPC/LOD/CMP/PST)에 추가. → Change Log 참조.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>P1 Mechanism은 모두 Prediction(Setup→Possible Observation) 성격이며 확정 인과가 아니다.</t>
         </is>
@@ -6479,7 +6785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -6674,177 +6980,189 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Axis: Lateral(Lead/Trail) [P7 계승] · AP(Anterior/Posterior) [Foot용 P1 신설]. 두 축 독립 — Lead(리드측 좌우)와 Anterior(전족부 전후)를 혼동 금지. [Ref: 좌우 / 전후 압력분포]</t>
+          <t>Axis: Lateral(Lead/Trail) [P7 계승] · AP(Anterior/Posterior) [Foot용 P1 신설]. 두 축 독립 — Lead(리드측 좌우)와 Anterior(전족부 전후)를 혼동 금지. Alias: Anterior=Forefoot, Posterior=Rearfoot(가독성용, 표준 축은 Anterior/Posterior). [Ref: 좌우 / 전후 압력분포]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
+          <t>★ Axis 통일 원칙</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Anterior/Posterior · Medial/Lateral · Superior/Inferior · Internal/External 등 해부학 축은 전 Object(Foot·Pelvis·Thorax·Spine 등)에 공통 재사용한다. 직관적 별칭(Forefoot/Rearfoot·Inside/Outside·High/Low)은 Alias로만 두고 Knowledge Graph의 표준 축 용어를 우선한다. → 'DOH Coordinate System' 시트 참조.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
           <t>Hand (P7 계승)</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Axis: Direction(Forward/Backward) · Height(High/Low) · Distance(Close/Far, Torso 기준) · Lateral(In/Out) · Depth(Deep/Shallow, Thorax 기준). P7 표준 그대로.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr"/>
-      <c r="B19" s="6" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr"/>
+      <c r="B20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>── Coordinate Reference Vocabulary (Axis 기준점) ──</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>Height (High / Low)</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>척추각 / 몸통·어깨 높이 기준</t>
-        </is>
-      </c>
+      <c r="B21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Tilt-Sagittal (Anterior / Posterior)</t>
+          <t>Height (High / Low)</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>골반 시상면 경사(전방/후방) 기준. 요추 만곡과 연동.</t>
+          <t>척추각 / 몸통·어깨 높이 기준</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Rotation (Open / Closed)</t>
+          <t>Tilt-Sagittal (Anterior / Posterior)</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Target Line 기준 (P7 계승)</t>
+          <t>골반 시상면 경사(전방/후방) 기준. 요추 만곡과 연동.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Elbow Rotation (Out / In)</t>
+          <t>Rotation (Open / Closed)</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>전완 외회전/내회전(External/Internal) 기준</t>
+          <t>Target Line 기준 (P7 계승)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Foot Angle (Toe-Out / Toe-In)</t>
+          <t>Elbow Rotation (Out / In)</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>발끝 외향/내향(External/Internal) 기준</t>
+          <t>전완 외회전/내회전(External/Internal) 기준</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Pressure Lateral (Lead / Trail)</t>
+          <t>Foot Angle (Toe-Out / Toe-In)</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>좌우 압력분포 기준 (P7 계승)</t>
+          <t>발끝 외향/내향(External/Internal) 기준</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Pressure AP (Anterior / Posterior)</t>
+          <t>Pressure Lateral (Lead / Trail)</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>발 전후 압력분포 기준(전족부/후족부). ※ Target Line의 Forward/Backward와 혼동 금지.</t>
+          <t>좌우 압력분포 기준 (P7 계승)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
+          <t>Pressure AP (Anterior / Posterior)</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>발 전후 압력분포 기준(전족부/후족부). ※ Target Line의 Forward/Backward와 혼동 금지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
           <t>Shaft Lean (Forward / Backward)</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Target Line 기준 (P7 Hand Direction과 동일 좌표)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr"/>
-      <c r="B29" s="6" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr"/>
+      <c r="B30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>── Mechanism Categories (P1) ──</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>ROT / PRS / ARM / CLB / SPC / LOD / CMP / PST</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>P7 카테고리 그대로 재사용.</t>
-        </is>
-      </c>
+      <c r="B31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>GRP (신규)</t>
+          <t>ROT / PRS / ARM / CLB / SPC / LOD / CMP / PST</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Grip — 양손 그립 방향 조합이 팔 연결성·페이스·코킹에 미치는 영향. P1에서 신설. (P7 PST 신설 선례와 동일 방식)</t>
+          <t>P7 카테고리 그대로 재사용(P7 LOCK, 약어 유지).</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr"/>
-      <c r="B33" s="6" t="inlineStr"/>
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>Grip (신규)</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>양손 그립 방향 조합이 팔 연결성·페이스·코킹에 미치는 영향. P1에서 신설(약어 없이 풀네임 'Grip'). P7 PST 신설 선례와 동일 방식. ※ 차기 Dictionary Refactoring에서 P7 카테고리도 풀네임 통일 검토 제안.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr"/>
+      <c r="B34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>⑦ Feature 신설 3원칙(P7 계승) + Information Gain 우선</t>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>새 Feature는 ①Observation이 다른가 ②새 Chain/Branch를 생성하는가 ③새 추론정보(Information Gain)를 주는가 를 모두 만족할 때만 만든다. DOH는 Feature 개수가 아니라 Knowledge 정보량을 늘리는 프로젝트다. 애매하면 임의 결정 없이 질문 후 진행한다.</t>
         </is>
@@ -6856,6 +7174,447 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Axis (표준 용어)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>반대극</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Alias (직관 표현)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Attribute 의미</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Used By (Object)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Coordinate Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Anterior</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Forefoot / Rearfoot (Foot Pressure)</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>앞(전방) / 뒤(후방)</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Foot Pressure, Pelvis Tilt, (향후 Thorax·Spine Translation/Tilt)</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>시상면(Sagittal) 전후</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>High / Low</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>위 / 아래</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Shoulder Height, Hand Height</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>척추각 / 몸통·어깨 높이</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Medial</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Lateral</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Inside / Outside</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>정중선 안쪽 / 바깥쪽</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Foot, Knee (위치)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>신체 정중선(Midline) 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>In / Out (회전)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>내회전 / 외회전</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Elbow Rotation, Hip Rotation, Foot Angle(Toe-In/Toe-Out)</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>회전축(장축) 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>좌 / 우 (타깃측/반대측)</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>리드측 / 트레일측</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Pressure(Lateral), Shoulder·Elbow Side</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>좌우(타깃 기준)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>목표선 대비 열림 / 닫힘</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Pelvis Rotation, Thorax Rotation, Club Face (P7)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Target Line</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Forward</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Backward</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>타깃 방향 / 반대</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Hand Direction (P7), Shaft Lean (P1/P7)</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Ball / Target Line</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Shallow</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>깊음 / 얕음</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Hand Depth (P7)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Thorax(몸 회전) 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Close To Body</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Far From Body</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Near / Far</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>몸에 가까움 / 멂</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Hand Distance (P7)</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Torso(몸) 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Steep</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>가파름 / 수평</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Shaft Plane</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>스윙 플레인</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Excessive</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Insufficient</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Too Much / Too Little</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>과다 / 부족</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Magnitude Modifier (전 Object 공통)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>정상범위(Reference) 대비</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>── DOH Coordinate System (Axis Master Reference) ── P1~P8 전 Object가 공유하는 좌표축 표준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>원칙: Axis(표준 용어)는 전 Object에 재사용한다. Foot에만 쓰는 Forefoot/Rearfoot 같은 표현은 Alias로만 두고, 표준 축 용어(Anterior/Posterior 등)를 Knowledge Graph의 canonical 값으로 사용한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>직관성보다 좌표계 일관성을 우선한다 — 예: Pelvis Tilt·Foot Pressure·Thorax Translation이 모두 Anterior/Posterior 축을 공유하므로 P2~P8에서 축을 새로 정의할 필요가 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>혼동 방지: Medial/Lateral(위치, 정중선) ≠ Internal/External(회전) ≠ Forward/Backward(Target Line) ≠ Lead/Trail(좌우). In/Out 표현은 문맥에 따라 회전(Internal/External) 또는 Target Line(Club Path) 중 하나로만 사용한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Attribute(방향극) + Magnitude(Excessive/Insufficient)로 Feature를 구성한다. 예: Pelvis Tilt(Object) + Anterior(Axis 극) + Excessive(Magnitude).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7072,7 +7831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7481,7 +8240,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8528,422 +9287,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>First Found</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Repeated</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Example / Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Flat Body Rotation</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>몸통이 수직 회전보다 수평 회전 성향을 더 많이 보이는 회전 패턴. 흉추 신전 부족과 함께 나타나며 팔이 과도하게 안쪽으로 이동하기 쉽다.</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Pelvis Tilt Posterior Excessive</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr"/>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Posterior Tilt → Flat Body Rotation → Inside Takeaway / Deep Hands. 반복 시 Biomechanical Concept 승격 검토.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Grip Match</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>리드 손과 트레일 손의 그립 방향이 서로 생체역학적으로 대응하는 정도(Strong/Weak/Neutral Match). 관용/상위 개념.</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Weak/Strong Grip Match</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Strong/Weak Grip Match Core Feature의 상위 개념. Naming 관용명 유지.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Clubhead Drag</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>어드레스·초기 스윙에서 클럽헤드가 손보다 과도하게 뒤처진 상태. 이후 Early Release·팔 보상 유발 가능.</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Shaft Lean Backward</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Shaft Lean Backward → Clubhead Drag → Early Release / Arm Dominant Pattern.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Arm Clearance</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>팔이 몸통과 간섭 없이 자연스럽게 움직일 수 있는 공간. 체형·흉곽 두께·셋업 자세에 영향.</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Deep Thorax (Setup Influence)</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Deep Thorax → Reduced Arm Clearance → Lead Arm Lift/Outside. Anthropometry 해석 보조.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Balance Recovery Strategy</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>초기 균형이 무너진 상태에서 반대 방향으로 압력·자세를 이동시켜 균형을 회복하려는 보상 전략.</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Foot Pressure (AP)</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Foot Pressure Anterior/Posterior의 Branch 분기 원인. Pressure·Posture·Rotation에서 반복 예상.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Compensatory Setup</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>신체 구조·가동성을 보상하기 위해 의도적으로 일반 기준과 다른 셋업을 사용하는 전략.</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Asymmetrical Foot Angle</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>좌우 발각도 비대칭 등. ④ 계층: 체형형 vs 습관형 구분과 연결.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Thorax Dominant Rotation</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>골반 회전이 제한될 때 흉곽 회전 의존도가 증가하는 회전 배분 패턴.</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Pelvis Tilt Anterior Excessive</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Anterior Tilt → Limited Pelvis Rotation → Thorax Dominant Rotation. 반복 시 승격 검토.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Movement Environment</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>P1 Setup이 정의하는, 특정 움직임이 발생하기 쉬운 초기 조건/움직임 편향(Initial Condition·Movement Bias). 확정 인과가 아닌 Prediction 대상.</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>P1 – 전체 Setup Feature</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>DOH 해석 철학(Knowledge Structure). P1 전 Feature의 상위 프레임. 반복성 확인 후 Standard 승격 검토.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Reverse Pivot</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>백스윙에서 체중·상체 축이 목표측(리드측)에 남아 정상과 반대로 기우는 축 패턴. 골프 관용명.</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Shoulder/APT/Lead Pressure</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>candidate-observation</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>다운스윙 보상이 매우 다양 → 단정 금지, P5~P7 검증. 관용명 유지.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Flat Shaft / Steep Shaft (Backswing)</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>백스윙 중 샤프트 플레인이 정상보다 수평(Flat)/수직(Steep)한 상태.</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Grip Match / Toe-In</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>candidate-observation</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>P4~P6 Observation. Shaft Plane 축. P6 Steep Shaft(P7 참조)와 Phase 구분.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Excessive Hip Depth</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>백스윙에서 엉덩이가 뒤로 과도하게 빠져 깊이가 증가한 상태(Early Extension 역방향).</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Foot Pressure Anterior</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr"/>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>candidate-observation</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Balance Recovery A 결과. P4 검증.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Balance Loss</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>후방/불안정 균형으로 자세 안정성이 무너지는 상태.</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>P1 – Foot Pressure Posterior</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>candidate-observation</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>P2~P4 검증. 반복성 확인 후 구조화.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>── DOH Candidate Concepts ── (검증 대기 공간 / Holding Area)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>⑤ 원칙: 새 Concept·해석 철학·Knowledge Structure·Feature화 애매 항목은 즉시 Feature화하지 않고 여기 먼저 등록. Repeated는 최초 등록 시 공백.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Promotion Rule: 3회 이상 반복 또는 2개 이상 Position(P1~P8)에서 재사용될 때 Feature/Biomechanical/Dictionary/Knowledge Structure 중 적절한 위치로 승격 검토.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>AI 판단 순서: ①기존 Dictionary ②기존 Feature ③기존 Biomechanical Concept ④새 Concept ⑤새 Knowledge Structure. 확신 없으면 Candidate 유지(삭제보다 보류).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: P1 Stage 2 — 심화 Chain(Medium) 5건 + Coaching/Biomech/Candidate 추가 + Field Observation 시트
사용자 추가 요청 반영:
- Foot Pressure Anterior/Posterior·Foot Angle Toe-Out/In·Lead Pressure에
  [Medium Confidence] 심화 Chain 추가(팔주도·Inside Delivery·Flying Elbow·
  Positive AoA·Hip Stability 등). Mechanism 56→68(재사용 우선).
- Coaching Knowledge +2 (Excessive Toe-Out/Toe-In Stance 보상 해석)
- Biomechanical Concepts +2 (Thoracic Compensation Strategy, Hip Internal Rotation Lock)
- Candidate: Compensatory Setup→Compensation Setup 통합 + Structural Compensation 신규
- 신규 시트 DOH Field Observation (레슨 현장 반복 관찰 DB, 승격 후보)
- 규칙 유지: Hook/Draw/Fat 등 결과는 Evidence Layer 관리, downstream 신규 노드는 관찰 대기 목록

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WzgekrgM9UsJ1Lha7AccVR
</commit_message>
<xml_diff>
--- a/DOH_P1.xlsx
+++ b/DOH_P1.xlsx
@@ -19,9 +19,10 @@
     <sheet name="DOH Candidate Concepts" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="DOH Biomechanical Concepts" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="DOH Coaching Knowledge" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Derived Parameters" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="DOH Change Log" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Todo" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="DOH Field Observation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Derived Parameters" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="DOH Change Log" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Todo" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1774,7 +1775,32 @@
 (하체의 저항이 감소하면 상·하체가 함께 회전하기 쉬워진다.)
  ↓
 Excessive Body Rotation (P4) [Candidate]
-※ Pattern Dependent</t>
+※ Pattern Dependent
+[Medium Confidence]  ※ Thoracic Compensation Strategy (Biomechanical Concept 참조)
+Foot Angle Toe-Out Excessive (P1)
+ ↓
+Excessive Toe-Out Often Accompanies Limited Thoracic Rotation As A Compensation.
+(과도한 발끝 벌림은 제한된 흉추 회전을 보상하려는 셋업으로 동반되는 경우가 많다.)
+ ↓
+Reduced Thoracic Rotation (P4) [예측·검증필요]
+── Branch (분기) ──
+The Player Chooses A Vertical Arm Motion Strategy.
+(팔을 보다 수직적으로 들어 올리는 전략을 선택한다.)
+ ↓
+Reduced Horizontal Rotation Promotes Vertical Arm Motion.
+(수평 회전이 제한되면 팔의 수직 움직임이 증가한다.)
+ ↓
+Flying Elbow (P4) [예측·검증필요]
+ ↓
+A Raised Trail Elbow Sets The Club Across The Line At The Top.
+(트레일 팔꿈치가 들리면 탑에서 클럽이 크로스 라인으로 놓인다.)
+ ↓
+Across The Line (P4) [예측·검증필요]  ※ = Cross Line
+ ↓
+An Across-The-Line Position Steepens The Downswing Shaft.
+(크로스 라인 포지션은 다운스윙 샤프트를 가파르게 만든다.)
+ ↓
+Steep Shaft (P6) [예측·검증필요]</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1931,25 @@
 (팔의 수직 움직임은 더욱 가파른 샤프트를 만든다.)
  ↓
 Steep Shaft (P4~P6) [예측·검증필요]
-※ Pattern Dependent</t>
+※ Pattern Dependent
+[Medium Confidence]  ※ Hip Internal Rotation Lock (Biomechanical Concept 참조)
+Foot Angle Toe-In Excessive (P1)
+ ↓
+The Toe-In Setup Maintains Hip Internal Rotation Restriction.
+(안짱걸음 셋업은 고관절 내회전 제한을 지속시킨다.)
+ ↓
+Hip Internal Rotation Restricted (P1~P4) [Reference / Mobility]
+ ↓
+Restricted Hip Internal Rotation Reduces Lateral Hip Stability.
+(고관절 내회전 제한은 고관절 외측 안정성을 감소시킨다.)
+ ↓
+Reduced Hip Stability (P4) [Candidate]
+── Branch (분기) ──
+The Player Chooses A Different Compensation Strategy During The Backswing.
+(백스윙에서 선택된 보상 전략이 이후 Chain을 결정한다.)
+ ↓
+Spin-Out (P6) / Pelvic Slide (P4) [Candidate] / Sway (P2~P4)
+※ Pattern Dependent (Lead Knee Collapse 동반 가능 → Field Observation 참조)</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2089,24 @@
 (백스윙에서 균형을 회복하려 압력을 뒤꿈치로 이동시킨다.)
  ↓
 Heel Pressure At Top (P4) [예측·검증필요]
-※ Balance Recovery Strategy B (보상)</t>
+※ Balance Recovery Strategy B (보상)
+[Medium Confidence]
+Foot Pressure Anterior Excessive (P1)
+ ↓
+Excessive Foot Balance Bias Reduces Available Rotation.
+(중립을 벗어난 발 균형은 가용 회전량을 감소시킨다.)
+ ↓
+Reduced Thoracic Rotation (P4) [예측·검증필요]
+ ↓
+Reduced Thoracic Rotation Shifts The Takeaway Toward Arm-Dominant Motion.
+(흉추 회전 감소는 테이크어웨이를 팔 주도로 이동시킨다.)
+ ↓
+Arm Dominant Takeaway (P2) [예측·검증필요]
+ ↓
+An Arm-Dominant Takeaway Leaves The Clubface Open.
+(팔 주도의 테이크어웨이는 페이스를 열린 채로 둔다.)
+ ↓
+Club Face Open (P4) [예측·검증필요]</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2238,25 @@
 (백스윙에서 균형을 회복하려 압력을 전족부로 이동시킨다.)
  ↓
 Toe Pressure During Backswing (P4) [예측·검증필요]
-※ Balance Recovery Strategy (보상)</t>
+※ Balance Recovery Strategy (보상)
+[Medium Confidence]
+Foot Pressure Posterior Excessive (P1)
+ ↓
+Heel-Ward Pressure Bias Directs The Early Club Path Inside.
+(후족부 압력 성향은 초기 클럽 경로를 안쪽으로 유도한다.)
+ ↓
+Inside Takeaway (P2) [예측·검증필요]
+ ↓
+An Inside Takeaway Promotes An Inside Club Delivery.
+(인사이드 테이크어웨이는 인사이드 클럽 전달을 유도한다.)
+ ↓
+Inside Club Delivery (P5~P6) [Candidate]
+ ↓
+An Inside, Shallow Delivery Tends To Produce A Positive Attack Angle.
+(인사이드·얕은 전달은 양(+)의 어택앵글 경향을 만든다.)
+ ↓
+Positive Attack Angle Tendency (P6) [Candidate · Parameter]
+※ Hook / Draw / Fat 등 결과는 Feature Chain이 아니라 Evidence Layer(Evidence Matrix)에서 관리</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2384,20 @@
 (백스윙 동안 압력이 리드측에 남아 있다.)
  ↓
 Reverse Pivot (P4) [예측·검증필요]
-※ ② Hold Strategy</t>
+※ ② Hold Strategy
+[Medium Confidence]
+Lead Pressure Excessive (P1)
+ ↓
+Pre-Set Lead Pressure Can Promote A Steeper Shaft Delivery.
+(어드레스 리드측 선하중은 더 가파른 샤프트 전달을 유도할 수 있다.)
+ ↓
+Steep Shaft Delivery (P5~P6) [예측·검증필요]
+ ↓
+A Steep Delivery With Rearward Weight Tends To Produce A Positive Attack Angle.
+(뒤에 남은 체중과 가파른 전달은 양(+)의 어택앵글 경향을 만든다.)
+ ↓
+Positive Attack Angle Tendency (P6) [Candidate · Parameter]
+※ Pattern Dependent</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2524,17 +2616,17 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Compensatory Setup</t>
+          <t>Compensation Setup</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>신체 구조·가동성을 보상하기 위해 의도적으로 일반 기준과 다른 셋업을 사용하는 전략.</t>
+          <t>골퍼가 신체 제한을 보상하기 위해 (무의식적으로) 일반 기준과 다른 셋업을 선택하는 전략.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>P1 – Asymmetrical Foot Angle</t>
+          <t>P1 – Asymmetrical Foot Angle / Toe-Out / Toe-In</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
@@ -2545,87 +2637,122 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>좌우 발각도 비대칭 등. ④ 계층: 체형형 vs 습관형 구분과 연결. P2~P8에서 반복 예상.</t>
+          <t>Toe-Out·Toe-In·Wide Stance 등 다양한 셋업에 적용. ④ 계층: 체형형 vs 습관형 구분과 연결. (기존 'Compensatory Setup'을 이 명칭으로 통합)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Movement Environment</t>
+          <t>Structural Compensation</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>P1 Setup이 정의하는, 특정 움직임이 발생하기 쉬운 초기 조건/움직임 편향(Initial Condition·Movement Bias). 확정 인과가 아닌 Prediction 대상.</t>
+          <t>신체 구조 또는 가동성 제한으로 인해 셋업 자체가 보상 형태로 형성되는 현상(전략 선택이 아닌 구조적 결과).</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>P1 – 전체 Setup Feature</t>
+          <t>P1 – Toe-Out / Spine Tilt / Shoulder Tilt</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr"/>
       <c r="E7" s="7" t="inlineStr">
         <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Compensation Setup(전략적 선택)과 구분되는 구조 기인형. Toe-Out·Spine Tilt·Shoulder Tilt 등.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Movement Environment</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>P1 Setup이 정의하는, 특정 움직임이 발생하기 쉬운 초기 조건/움직임 편향(Initial Condition·Movement Bias). 확정 인과가 아닌 Prediction 대상.</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>P1 – 전체 Setup Feature</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
           <t>Candidate (승격 검토중)</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>DOH 해석 철학(Knowledge Structure). P1 전 13 Feature의 상위 프레임. ★사용자 승격 승인 — 반복성 확인 후 Knowledge Structure로 승격.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>── DOH Candidate Concepts ── (검증 대기 공간 / Holding Area) · 반복성 있는 개념만 유지(6개)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>⑤ 원칙: 새 Concept·해석 철학·Knowledge Structure·Feature화 애매 항목은 즉시 Feature화하지 않고 여기 먼저 등록. Repeated는 최초 등록 시 공백.</t>
+          <t>── DOH Candidate Concepts ── (검증 대기 공간 / Holding Area) · 반복성 있는 개념만 유지(7개)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
+          <t>⑤ 원칙: 새 Concept·해석 철학·Knowledge Structure·Feature화 애매 항목은 즉시 Feature화하지 않고 여기 먼저 등록. Repeated는 최초 등록 시 공백.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
           <t>Promotion Rule: 3회 이상 반복 또는 2개 이상 Position(P1~P8)에서 재사용될 때 Feature/Biomechanical/Dictionary/Knowledge Structure 중 적절한 위치로 승격 검토.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>── 관찰 노드 대기 목록 (Concept 아님 · P2~P4 표준화 대기 · 단일 출현이라 Candidate 미등록) ──</t>
-        </is>
-      </c>
+      <c r="A13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Reverse Pivot — 다운스윙 보상 다양, P5~P7 검증 대상(관용명). / Flat·Steep Shaft (Backswing) — Shaft Plane 축, P4~P6 Observation.</t>
+          <t>── 관찰 노드 대기 목록 (Concept 아님 · P2~P4 표준화 대기 · 단일/소수 출현이라 Candidate 미등록) ──</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Excessive Hip Depth — Balance Recovery A 결과, P4 검증. / Balance Loss — P2~P4 검증. / Clubhead Drag — 현재 P1 단일 출현, P2~P4에서 반복되면 Candidate 승격 검토. / Thorax Dominant Rotation — 현재 APT 단일 출현, 반복 시 승격 검토.</t>
+          <t>Reverse Pivot / Flat·Steep Shaft(Backswing) / Excessive Hip Depth / Balance Loss / Clubhead Drag / Thorax Dominant Rotation.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>→ 위 노드들은 P2~P4 진행 중 반복 확인되면 Candidate Concepts로 정식 등록한다(살아남는 개념만 승격).</t>
+          <t>Stage2 심화 Chain 신규 노드: Flying Elbow(P4) / Across The Line(=Cross Line, P4) / Thoracic Hyperextension(P4) / Arm Dominant Takeaway(P2) / Inside Club Delivery(P5~P6) / Reduced Hip Stability(P4) / Pelvic Slide(P4) / Lead Knee Collapse(P4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Positive Attack Angle Tendency(P6) — Attack Angle은 P5~P8 Derived Parameter 계열(Derived Parameters 시트 참조). P1에서는 '경향(Tendency)'만 예측.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>→ 위 노드들은 P2~P4 진행 중 반복 확인되면 Candidate/Feature/Biomechanical로 정식 승격한다(살아남는 개념만 승격).</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2803,22 +2930,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Thoracic Compensation Strategy</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>제한된 흉추 회전을 발 위치·척추 신전·팔 구조 등으로 보상하는 운동 전략.</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-Out Excessive (P1), Flying Elbow, Thoracic Hyperextension</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>AI는 Toe-Out을 독립 문제로 판단하지 않고 흉추 제한에 대한 보상 전략인지 함께 해석한다.</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>── DOH Biomechanical Concepts ── Feature가 아닌, Mechanism 설명에 반복 등장하는 생체역학 언어.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>목적: 동일한 생체역학 개념을 항상 동일한 언어로 설명. AI는 Feature/Mechanism 생성 시 이 페이지를 우선 참고.</t>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Hip Internal Rotation Lock</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>고관절이 내회전 상태로 고정되어 외측 안정성이 감소하는 생체역학적 상태.</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-In Excessive (P1), Lead Knee Collapse, Spin-Out, Pelvic Slide</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>AI는 Toe-In 셋업을 Hip Stability와 연결하여 이후 회전 전략·보상 패턴을 추론한다.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>── DOH Biomechanical Concepts ── Feature가 아닌, Mechanism 설명에 반복 등장하는 생체역학 언어.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>목적: 동일한 생체역학 개념을 항상 동일한 언어로 설명. AI는 Feature/Mechanism 생성 시 이 페이지를 우선 참고.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>승격 근거: Thoracic Extension·Hip Rotation·Lumbar Lordosis·Center Of Pressure는 P1 Mechanism에서 반복 등장하여 등록.</t>
         </is>
@@ -2835,7 +3006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3218,22 +3389,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Excessive Toe-Out Stance</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Excessive Toe-Out Stance는 흉추 회전이 제한된 골퍼에게서 자주 관찰되는 보상성 셋업이다. 많은 골퍼는 부족한 흉추 회전을 보상하기 위해 자연스럽게 발끝을 바깥쪽으로 벌리는 전략을 선택한다. 이러한 골퍼는 백스윙 Top(P4)에서 Flying Elbow, Cross Line(Across The Line), Thoracic Hyperextension이 함께 나타나는 경우가 많다. Toe-Out 자체를 문제로 판단하기보다 제한된 Thoracic Rotation에 대한 보상 전략인지 먼저 확인해야 한다.</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>── DOH Coaching Knowledge ── Feature/Mechanism/Observation만으로 설명하기 어려운 레슨 경험·조건부 해석·전략·예외.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>AI는 Feature/Mechanism을 우선 사용하며, 충분히 설명되지 않을 때만 Coaching Knowledge를 참고해 설명·피드백·질문·전략을 생성한다.</t>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Excessive Toe-In Stance</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Excessive Toe-In Stance는 고관절이 내회전된 상태에서 셋업되는 골퍼에게 자주 관찰된다. 이러한 골퍼는 고관절 외측 안정성이 감소하고, 둔근과 외전근의 기능 저하가 함께 나타나는 경우가 많다. 결과적으로 Spin-Out, Pelvic Slide, Sway, Lead Knee Collapse가 동반될 가능성이 높다. Toe-In 자체보다 Hip Internal Rotation과 Hip Stability를 함께 평가해야 한다.</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>── DOH Coaching Knowledge ── Feature/Mechanism/Observation만으로 설명하기 어려운 레슨 경험·조건부 해석·전략·예외.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>AI는 Feature/Mechanism을 우선 사용하며, 충분히 설명되지 않을 때만 Coaching Knowledge를 참고해 설명·피드백·질문·전략을 생성한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>※ Coaching Knowledge는 Observation이 아니며 Feature를 생성하지 않는다. AI의 최종 판단 근거가 아니라 Explanation/Coaching/Strategy/Exception 제공용이다.</t>
         </is>
@@ -3245,6 +3460,190 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Frequency</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Related Features</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Toe-Out 골퍼는 Flying Elbow를 매우 자주 동반한다.</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Very Common</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-Out Excessive (P1), Flying Elbow</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>레슨 경험 기반</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Toe-Out 골퍼는 Thoracic Hyperextension으로 회전을 보상하는 경우가 많다.</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-Out Excessive (P1), Thoracic Hyperextension</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>반복 관찰</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Toe-In 골퍼는 Spin-Out과 Pelvic Slide를 자주 동반한다.</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-In Excessive (P1), Spin-Out, Pelvic Slide</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>레슨 경험 기반</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Toe-In 골퍼는 Lead Knee Collapse가 함께 나타나는 경우가 많다.</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-In Excessive (P1), Lead Knee Collapse</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>반복 관찰</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>── DOH Field Observation ── 논문·Feature·Mechanism이 아니라, 실제 레슨에서 반복 관찰한 경험을 축적하는 데이터베이스.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>현재는 AI 추론에 직접 사용하지 않는다. 향후 반복성·재사용성이 검증되면 Coaching Knowledge / Mechanism / Candidate Concepts / Feature로 승격할 수 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>형식: Observation · Frequency(Very Common/Common/Occasional) · Confidence · Related Features · Notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Frequency·Confidence는 레슨 경험 기반의 주관적 추정치이며, 확정 인과나 Observation Feature가 아니다.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3313,13 +3712,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3585,7 +3984,7 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>── P7 Standard 개선 제안 (참고용, 미변경) ──</t>
+          <t>── Stage 2 추가 (심화 Chain + Field Observation) ──</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr"/>
@@ -3594,66 +3993,160 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>제안 1 — ★승인</t>
+          <t>Mechanism Added (+12)</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Naming Rule에 'Side 배치 관례' 명문화</t>
+          <t>심화 Chain Mechanism</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>P1에서 'Object Axis [Side] [Attribute]' 관례를 명문화. 사용자 승인 — 차기 Dictionary Refactoring 시 P7 Naming Rule에도 역반영 예정. (현재 P7 미변경)</t>
+          <t>Foot Pressure Anterior→Arm Dominant Takeaway→Club Face Open / Posterior→Inside Delivery→Positive AoA / Toe-Out→Reduced Thoracic→Flying Elbow→Across The Line→Steep Shaft / Lead Pressure→Steep Delivery→Positive AoA / Toe-In→Hip IR Restricted→Reduced Hip Stability→Spin-Out·Pelvic Slide·Sway. 총 56→68. 재사용: 발 균형→회전·Heel-Ward Inside·Vertical Arm·Branch 표준문장.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>제안 2 — 보류</t>
+          <t>Coaching Added (+2)</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Movement Environment를 Knowledge Structure로 승격</t>
+          <t>Toe-Out / Toe-In Stance</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>'Setup=Movement Environment' 프레임을 Knowledge Structure로 승격 검토. ★사용자 승인 — 반복성 확인(P2~P4) 후 정식 승격. (현재 Candidate 유지)</t>
+          <t>Toe-Out=흉추 회전 제한 보상성 셋업(Flying Elbow·Cross Line·Thoracic Hyperextension 동반). Toe-In=고관절 내회전·둔근/외전근 저하(Spin-Out·Pelvic Slide·Sway·Lead Knee Collapse 동반). (사용자 제공)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>제안 3 — 보류</t>
+          <t>Candidate 정리(+2, 병합1)</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Phase-Distinguished Pair 명시 필드</t>
+          <t>Compensation Setup / Structural Compensation</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>사용자 보류: Knowledge Graph가 자동 연결해야 하며 문서에 Pair를 쓰면 중복 관리가 됨. P2~P4 진행 후 재판단. (미반영)</t>
+          <t>기존 'Compensatory Setup'을 'Compensation Setup'으로 통합(중복 방지), 'Structural Compensation'(구조 기인형) 신규. Candidate 6→7.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
+          <t>Biomechanical Added (+2)</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Thoracic Compensation Strategy / Hip Internal Rotation Lock</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Toe-Out/Toe-In의 상위 생체역학 해석. AI가 셋업을 독립 문제가 아닌 보상 전략/구조로 해석하도록 함. (사용자 제공)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>신규 시트</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>DOH Field Observation</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>레슨 현장 반복 관찰 축적 DB(4건). AI 직접 사용 안 함 — 반복성 검증 후 Coaching/Mechanism/Candidate/Feature 승격 후보. (사용자 제안)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>── P7 Standard 개선 제안 (참고용, 미변경) ──</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr"/>
+      <c r="C22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>제안 1 — ★승인</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Naming Rule에 'Side 배치 관례' 명문화</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>P1에서 'Object Axis [Side] [Attribute]' 관례를 명문화. 사용자 승인 — 차기 Dictionary Refactoring 시 P7 Naming Rule에도 역반영 예정. (현재 P7 미변경)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>제안 2 — 보류</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Movement Environment를 Knowledge Structure로 승격</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>'Setup=Movement Environment' 프레임을 Knowledge Structure로 승격 검토. ★사용자 승인 — 반복성 확인(P2~P4) 후 정식 승격. (현재 Candidate 유지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>제안 3 — 보류</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Phase-Distinguished Pair 명시 필드</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>사용자 보류: Knowledge Graph가 자동 연결해야 하며 문서에 Pair를 쓰면 중복 관리가 됨. P2~P4 진행 후 재판단. (미반영)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
           <t>제안 4 — 보류</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Prediction vs Observed 태그</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>사용자 보류: P1 자체가 Prediction, P7이 Observation이므로 별도 태그 불필요할 수 있음. P2~P4 진행 후 재판단. (미반영)</t>
         </is>
@@ -3664,13 +4157,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3803,19 +4296,19 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>56문장(중복 검토·통합 완료, 58→56). ★재사용 Node/Branch 표준문장 표시.</t>
+          <t>68문장(기본 56 + Stage2 심화 Chain 12). 중복 검토·통합 완료. ★재사용 Node/Branch 표준문장 표시.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Setup Influence(Setup/Anthropometry/Mobility → Prediction)</t>
+          <t>Stage2 심화 Chain(Medium) 5 Feature + Field Observation</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -3825,7 +4318,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>계층 분리 반영.</t>
+          <t>Foot Pressure AP·Toe-Out/In·Lead Pressure 심화. DOH Field Observation 시트 신설.</t>
         </is>
       </c>
     </row>
@@ -3837,7 +4330,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Candidate Concepts 통합 + 신규 등록</t>
+          <t>Setup Influence(Setup/Anthropometry/Mobility → Prediction)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -3847,7 +4340,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>중복 시트 통합. Repeated 공백.</t>
+          <t>계층 분리 반영.</t>
         </is>
       </c>
     </row>
@@ -3859,7 +4352,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Biomechanical Concepts 확장</t>
+          <t>Candidate Concepts 통합 + 신규 등록</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -3869,7 +4362,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Thoracic Extension 등 4항목 추가.</t>
+          <t>중복 시트 통합. Repeated 공백.</t>
         </is>
       </c>
     </row>
@@ -3881,7 +4374,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Coaching Knowledge 보존·표준화</t>
+          <t>Biomechanical Concepts 확장</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -3891,7 +4384,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>15항목. Category/Topic/Knowledge/Confidence.</t>
+          <t>Thoracic Extension 등 4항목 추가.</t>
         </is>
       </c>
     </row>
@@ -3903,7 +4396,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Evidence Layer/Matrix 구조(별점 보류)</t>
+          <t>Coaching Knowledge 보존·표준화</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -3913,19 +4406,19 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>P1 간접 연결 특성 명시.</t>
+          <t>15항목. Category/Topic/Knowledge/Confidence.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>P1 메인 시트: Core 13 Feature 6-섹션</t>
+          <t>Evidence Layer/Matrix 구조(별점 보류)</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -3935,7 +4428,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Dictionary 기준 문장 사용. Movement Environment 관점.</t>
+          <t>P1 간접 연결 특성 명시.</t>
         </is>
       </c>
     </row>
@@ -3947,7 +4440,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>규칙 적용: Chain 종료·Branch Mechanism·Confidence 3단계·Family·Fat/Thin 제거</t>
+          <t>P1 메인 시트: Core 13 Feature 6-섹션</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -3955,7 +4448,11 @@
           <t>done</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr"/>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Dictionary 기준 문장 사용. Movement Environment 관점.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -3965,7 +4462,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>DOH Change Log(Added 정리 + P7 개선 제안)</t>
+          <t>규칙 적용: Chain 종료·Branch Mechanism·Confidence 3단계·Family·Fat/Thin 제거</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -3973,31 +4470,27 @@
           <t>done</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>규칙 ⑥.</t>
-        </is>
-      </c>
+      <c r="D14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Evidence Matrix 별점 일괄 부여</t>
+          <t>DOH Change Log(Added 정리 + P7 개선 제안)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>todo</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>P1~P8 설계 완료 후 별도 세션.</t>
+          <t>규칙 ⑥.</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4502,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>HTML/JSON 변환</t>
+          <t>Evidence Matrix 별점 일괄 부여</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -4019,23 +4512,45 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>P1~P8 LOCK 후 일괄.</t>
+          <t>P1~P8 설계 완료 후 별도 세션.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>HTML/JSON 변환</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>P1~P8 LOCK 후 일괄.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
           <t>참고</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>작업 순서</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr"/>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Dictionary → Feature 6-섹션 → Evidence 별점 → HTML/JSON. 동일 의미=동일 문장.</t>
         </is>
@@ -4052,7 +4567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5679,43 +6194,379 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Reduced Thoracic Rotation Shifts The Takeaway Toward Arm-Dominant Motion.</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>흉추 회전 감소는 테이크어웨이를 팔 주도로 이동시킨다.</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr"/>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Foot Pressure Anterior Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. Reduced Thoracic Rotation→Arm Dominant Takeaway.</t>
+        </is>
+      </c>
+    </row>
     <row r="59">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>── DOH P1 Mechanism Dictionary ── (총 56문장)</t>
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>An Arm-Dominant Takeaway Leaves The Clubface Open.</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>팔 주도의 테이크어웨이는 페이스를 열린 채로 둔다.</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr"/>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Foot Pressure Anterior Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. →Club Face Open (P4).</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>An Inside Takeaway Promotes An Inside Club Delivery.</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>인사이드 테이크어웨이는 인사이드 클럽 전달을 유도한다.</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr"/>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Foot Pressure Posterior Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. →Inside Club Delivery(Candidate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>An Inside, Shallow Delivery Tends To Produce A Positive Attack Angle.</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>인사이드·얕은 전달은 양(+)의 어택앵글 경향을 만든다.</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr"/>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Foot Pressure Posterior Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. →Positive Attack Angle Tendency(Parameter).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Excessive Toe-Out Often Accompanies Limited Thoracic Rotation As A Compensation.</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>과도한 발끝 벌림은 제한된 흉추 회전을 보상하려는 셋업으로 동반되는 경우가 많다.</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr"/>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-Out Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. Structural/Thoracic Compensation. Toe-Out↔Limited Thoracic Rotation 동반.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>The Player Chooses A Vertical Arm Motion Strategy.</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>팔을 보다 수직적으로 들어 올리는 전략을 선택한다.</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr"/>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-Out Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. ★Branch 분기 문장(수직 팔 전략).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>A Raised Trail Elbow Sets The Club Across The Line At The Top.</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>트레일 팔꿈치가 들리면 탑에서 클럽이 크로스 라인으로 놓인다.</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr"/>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-Out Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. Flying Elbow→Across The Line(=Cross Line).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>An Across-The-Line Position Steepens The Downswing Shaft.</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>크로스 라인 포지션은 다운스윙 샤프트를 가파르게 만든다.</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr"/>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-Out Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. →Steep Shaft (P6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Pre-Set Lead Pressure Can Promote A Steeper Shaft Delivery.</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>어드레스 리드측 선하중은 더 가파른 샤프트 전달을 유도할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr"/>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. →Steep Shaft Delivery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>A Steep Delivery With Rearward Weight Tends To Produce A Positive Attack Angle.</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>뒤에 남은 체중과 가파른 전달은 양(+)의 어택앵글 경향을 만든다.</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr"/>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. →Positive Attack Angle Tendency(Parameter).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>The Toe-In Setup Maintains Hip Internal Rotation Restriction.</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>안짱걸음 셋업은 고관절 내회전 제한을 지속시킨다.</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr"/>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-In Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. Toe-In→Hip IR Restricted(Reference/Mobility).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>LOD</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Restricted Hip Internal Rotation Reduces Lateral Hip Stability.</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>고관절 내회전 제한은 고관절 외측 안정성을 감소시킨다.</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr"/>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Foot Angle Toe-In Excessive (P1)</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>P1 Stage2. →Reduced Hip Stability(Candidate). Hip Internal Rotation Lock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>── DOH P1 Mechanism Dictionary ── (총 68문장: 기본 56 + Stage2 심화 Chain 12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>③ 원칙: 동일 Mechanism 반복 시 재사용 우선. 새 Mechanism은 기존 Dictionary로 설명 불가할 때만 추가.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
         <is>
           <t>★재사용 Node: 'Vertical Arm Motion Promotes A Steeper Shaft Plane.'(Weak Grip Match/Toe-In) · 'Excessive Foot Balance Bias Reduces Available Rotation.'(Anterior/Posterior) · Branch 표준문장(Anterior/Lead Pressure).</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>★신규 카테고리 Grip: P1에서 신설(풀네임). P7 카테고리(ROT/PRS/ARM/CLB/SPC/LOD/CMP/PST)에 추가. → Change Log 참조.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
         <is>
           <t>중복 검토 완료: 의미 중복 2쌍 통합(발 균형→회전 / Branch 문장), APT-PPT 'Late Wrist Set' 오통합 분리(반대 원인), 'Steeper Arm Motion'→'Vertical Arm Motion' 정합. shoulder/elbow→Outside 등은 Object 상이로 유지.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>P1 Mechanism은 모두 Prediction(Setup→Possible Observation) 성격이며 확정 인과가 아니다.</t>
         </is>

</xml_diff>

<commit_message>
refactor: Cross Line 표준어 통일 + Compensation Setup 통합 확정
사용자 지시 반영:
- DOH Standard 표준어를 'Cross Line'으로 통일(Feature·Dictionary·Mechanism).
  'Across The Line'은 cross-reference(동의어)로만 유지(Mechanism Replaces 컬럼).
- 'Compensatory Setup'은 별도 Concept 미유지 → 'Compensation Setup'에 통합, cross-reference만.
- 신규 Concept는 Candidate/Field Observation으로 관리, 다중 Phase 재사용 확인 시에만 승격 제안.
- Evidence Matrix 별점은 그대로 미입력(구조만 유지).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WzgekrgM9UsJ1Lha7AccVR
</commit_message>
<xml_diff>
--- a/DOH_P1.xlsx
+++ b/DOH_P1.xlsx
@@ -945,7 +945,7 @@
 The Club Continues Moving After Arm Rotation Stops.
 (팔 회전이 멈춘 이후에도 클럽이 계속 이동한다.)
  ↓
-Across The Line (P4) [예측·검증필요]
+Cross Line (P4) [예측·검증필요]  ※ = Across The Line (cross-ref)
 ※ Pattern Dependent
 Flat Body Rotation (P2~P4)
  ↓
@@ -1792,12 +1792,12 @@
  ↓
 Flying Elbow (P4) [예측·검증필요]
  ↓
-A Raised Trail Elbow Sets The Club Across The Line At The Top.
-(트레일 팔꿈치가 들리면 탑에서 클럽이 크로스 라인으로 놓인다.)
- ↓
-Across The Line (P4) [예측·검증필요]  ※ = Cross Line
- ↓
-An Across-The-Line Position Steepens The Downswing Shaft.
+A Raised Trail Elbow Sets The Club In A Cross-Line Position At The Top.
+(트레일 팔꿈치가 들리면 탑에서 클럽이 크로스 라인 포지션에 놓인다.)
+ ↓
+Cross Line (P4) [예측·검증필요]  ※ = Across The Line (cross-ref)
+ ↓
+A Cross-Line Position Steepens The Downswing Shaft.
 (크로스 라인 포지션은 다운스윙 샤프트를 가파르게 만든다.)
  ↓
 Steep Shaft (P6) [예측·검증필요]</t>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Toe-Out·Toe-In·Wide Stance 등 다양한 셋업에 적용. ④ 계층: 체형형 vs 습관형 구분과 연결. (기존 'Compensatory Setup'을 이 명칭으로 통합)</t>
+          <t>Toe-Out·Toe-In·Wide Stance 등 다양한 셋업에 적용. ④ 계층: 체형형 vs 습관형 구분과 연결. (동의어 cross-reference: 구 'Compensatory Setup' → 별도 Concept 유지 안 함, 본 명칭으로 통합)</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Stage2 심화 Chain 신규 노드: Flying Elbow(P4) / Across The Line(=Cross Line, P4) / Thoracic Hyperextension(P4) / Arm Dominant Takeaway(P2) / Inside Club Delivery(P5~P6) / Reduced Hip Stability(P4) / Pelvic Slide(P4) / Lead Knee Collapse(P4).</t>
+          <t>Stage2 심화 Chain 신규 노드: Flying Elbow(P4) / Cross Line(P4, 표준어 · = Across The Line cross-ref) / Thoracic Hyperextension(P4) / Arm Dominant Takeaway(P2) / Inside Club Delivery(P5~P6) / Reduced Hip Stability(P4) / Pelvic Slide(P4) / Lead Knee Collapse(P4).</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Foot Pressure Anterior→Arm Dominant Takeaway→Club Face Open / Posterior→Inside Delivery→Positive AoA / Toe-Out→Reduced Thoracic→Flying Elbow→Across The Line→Steep Shaft / Lead Pressure→Steep Delivery→Positive AoA / Toe-In→Hip IR Restricted→Reduced Hip Stability→Spin-Out·Pelvic Slide·Sway. 총 56→68. 재사용: 발 균형→회전·Heel-Ward Inside·Vertical Arm·Branch 표준문장.</t>
+          <t>Foot Pressure Anterior→Arm Dominant Takeaway→Club Face Open / Posterior→Inside Delivery→Positive AoA / Toe-Out→Reduced Thoracic→Flying Elbow→Cross Line→Steep Shaft / Lead Pressure→Steep Delivery→Positive AoA / Toe-In→Hip IR Restricted→Reduced Hip Stability→Spin-Out·Pelvic Slide·Sway. 총 56→68. 재사용: 발 균형→회전·Heel-Ward Inside·Vertical Arm·Branch 표준문장.</t>
         </is>
       </c>
     </row>
@@ -4076,77 +4076,128 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>── P7 Standard 개선 제안 (참고용, 미변경) ──</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr"/>
-      <c r="C22" s="7" t="inlineStr"/>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>표준어 통일</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Cross Line</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>DOH Standard 표준어를 'Cross Line'으로 통일(사용자 지시). Feature·Dictionary·Mechanism 모두 Cross Line 사용. 'Across The Line'은 cross-reference(동의어)로만 유지(Mechanism Replaces 컬럼에 기록).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>제안 1 — ★승인</t>
+          <t>Concept 통합</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Naming Rule에 'Side 배치 관례' 명문화</t>
+          <t>Compensation Setup</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>P1에서 'Object Axis [Side] [Attribute]' 관례를 명문화. 사용자 승인 — 차기 Dictionary Refactoring 시 P7 Naming Rule에도 역반영 예정. (현재 P7 미변경)</t>
+          <t>'Compensatory Setup'은 별도 Concept로 유지하지 않고 'Compensation Setup'에 통합, cross-reference만 남김(사용자 지시).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>제안 2 — 보류</t>
+          <t>Concept 승격 정책</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Movement Environment를 Knowledge Structure로 승격</t>
+          <t>Candidate/Field 유지</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>'Setup=Movement Environment' 프레임을 Knowledge Structure로 승격 검토. ★사용자 승인 — 반복성 확인(P2~P4) 후 정식 승격. (현재 Candidate 유지)</t>
+          <t>신규 Concept는 Candidate/Field Observation으로 관리하고, 여러 Phase에서 반복·재사용성이 확인된 경우에만 DOH Standard 승격을 제안한다(사용자 지시).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>제안 3 — 보류</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Phase-Distinguished Pair 명시 필드</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>사용자 보류: Knowledge Graph가 자동 연결해야 하며 문서에 Pair를 쓰면 중복 관리가 됨. P2~P4 진행 후 재판단. (미반영)</t>
-        </is>
-      </c>
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>── P7 Standard 개선 제안 (참고용, 미변경) ──</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr"/>
+      <c r="C25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
+          <t>제안 1 — ★승인</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Naming Rule에 'Side 배치 관례' 명문화</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>P1에서 'Object Axis [Side] [Attribute]' 관례를 명문화. 사용자 승인 — 차기 Dictionary Refactoring 시 P7 Naming Rule에도 역반영 예정. (현재 P7 미변경)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>제안 2 — 보류</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Movement Environment를 Knowledge Structure로 승격</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>'Setup=Movement Environment' 프레임을 Knowledge Structure로 승격 검토. ★사용자 승인 — 반복성 확인(P2~P4) 후 정식 승격. (현재 Candidate 유지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>제안 3 — 보류</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Phase-Distinguished Pair 명시 필드</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>사용자 보류: Knowledge Graph가 자동 연결해야 하며 문서에 Pair를 쓰면 중복 관리가 됨. P2~P4 진행 후 재판단. (미반영)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
           <t>제안 4 — 보류</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Prediction vs Observed 태그</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>사용자 보류: P1 자체가 Prediction, P7이 Observation이므로 별도 태그 불필요할 수 있음. P2~P4 진행 후 재판단. (미반영)</t>
         </is>
@@ -4746,7 +4797,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>P1 신규. Late Wrist Set→Across The Line.</t>
+          <t>P1 신규. Late Wrist Set→Cross Line (표준어; = Across The Line).</t>
         </is>
       </c>
     </row>
@@ -6370,15 +6421,19 @@
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
+          <t>A Raised Trail Elbow Sets The Club In A Cross-Line Position At The Top.</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>트레일 팔꿈치가 들리면 탑에서 클럽이 크로스 라인 포지션에 놓인다.</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
           <t>A Raised Trail Elbow Sets The Club Across The Line At The Top.</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>트레일 팔꿈치가 들리면 탑에서 클럽이 크로스 라인으로 놓인다.</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="inlineStr"/>
       <c r="E64" s="7" t="inlineStr">
         <is>
           <t>Foot Angle Toe-Out Excessive (P1)</t>
@@ -6386,7 +6441,7 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>P1 Stage2. Flying Elbow→Across The Line(=Cross Line).</t>
+          <t>P1 Stage2. Flying Elbow→Cross Line (표준어; = Across The Line cross-ref).</t>
         </is>
       </c>
     </row>
@@ -6398,15 +6453,19 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
+          <t>A Cross-Line Position Steepens The Downswing Shaft.</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>크로스 라인 포지션은 다운스윙 샤프트를 가파르게 만든다.</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
           <t>An Across-The-Line Position Steepens The Downswing Shaft.</t>
         </is>
       </c>
-      <c r="C65" s="7" t="inlineStr">
-        <is>
-          <t>크로스 라인 포지션은 다운스윙 샤프트를 가파르게 만든다.</t>
-        </is>
-      </c>
-      <c r="D65" s="7" t="inlineStr"/>
       <c r="E65" s="7" t="inlineStr">
         <is>
           <t>Foot Angle Toe-Out Excessive (P1)</t>
@@ -6414,7 +6473,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>P1 Stage2. →Steep Shaft (P6).</t>
+          <t>P1 Stage2. Cross Line→Steep Shaft (P6).</t>
         </is>
       </c>
     </row>

</xml_diff>